<commit_message>
[refs #36200] Fixes to approval summary export.
</commit_message>
<xml_diff>
--- a/core/api/export/templates/approval_summary_template.xlsx
+++ b/core/api/export/templates/approval_summary_template.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Work/edw/ors-multilateralfund/core/api/export/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{48292208-5130-44DA-9346-E260766999CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE109C0F-ECC6-1F41-8653-EAE05C0DB67E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="28488" windowHeight="15420" xr2:uid="{EFCB9BCD-D7D4-4B7E-959C-9F2ED12FB513}"/>
+    <workbookView xWindow="780" yWindow="2800" windowWidth="28480" windowHeight="15420" xr2:uid="{EFCB9BCD-D7D4-4B7E-959C-9F2ED12FB513}"/>
   </bookViews>
   <sheets>
     <sheet name="Approval summary" sheetId="2" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Approval summary'!$B$1:$G$53</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -106,9 +109,6 @@
     <t>(ODP tonnes)</t>
   </si>
   <si>
-    <t>Funds reccommended (US $)</t>
-  </si>
-  <si>
     <t>HFC</t>
   </si>
   <si>
@@ -119,14 +119,18 @@
   </si>
   <si>
     <t xml:space="preserve">Summary  </t>
+  </si>
+  <si>
+    <t>Funds recommended (US$)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="#,##0;[Red]\-&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -263,18 +267,9 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -294,12 +289,21 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -320,9 +324,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -360,7 +364,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -466,7 +470,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -608,7 +612,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -618,31 +622,32 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{785D2C6E-8947-4B91-9DE2-B2934FDC0F4D}">
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:S38"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="1"/>
-    <col min="2" max="2" width="34.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" style="1" customWidth="1"/>
     <col min="8" max="12" width="8.6640625" style="1"/>
     <col min="13" max="13" width="28.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="40" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="28.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:19" ht="23.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="22" t="s">
-        <v>27</v>
+    <row r="1" spans="2:19" ht="23.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="18" t="s">
+        <v>26</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
@@ -650,136 +655,136 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
     </row>
-    <row r="2" spans="2:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="20" t="s">
+    <row r="2" spans="2:19" ht="18.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="C2" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="D2" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-    </row>
-    <row r="3" spans="2:19" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="18"/>
-      <c r="C3" s="17" t="s">
+      <c r="E2" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+    </row>
+    <row r="3" spans="2:19" ht="25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="15"/>
+      <c r="C3" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="2:19" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="12" t="s">
+    <row r="4" spans="2:19" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
       <c r="S4" s="3"/>
     </row>
-    <row r="5" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B5" s="7" t="s">
+    <row r="5" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="7">
-        <v>0</v>
-      </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="5">
-        <v>0</v>
-      </c>
-      <c r="F5" s="5">
-        <v>0</v>
-      </c>
-      <c r="G5" s="5">
+      <c r="C5" s="6">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="19">
+        <v>0</v>
+      </c>
+      <c r="F5" s="19">
+        <v>0</v>
+      </c>
+      <c r="G5" s="19">
         <v>0</v>
       </c>
       <c r="S5" s="3"/>
     </row>
-    <row r="6" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B6" s="7" t="s">
+    <row r="6" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="5">
-        <v>0</v>
-      </c>
-      <c r="F6" s="5">
-        <v>0</v>
-      </c>
-      <c r="G6" s="5">
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="19">
+        <v>0</v>
+      </c>
+      <c r="F6" s="19">
+        <v>0</v>
+      </c>
+      <c r="G6" s="19">
         <v>0</v>
       </c>
       <c r="S6" s="3"/>
     </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B7" s="7" t="s">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7">
-        <v>0</v>
-      </c>
-      <c r="E7" s="5">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5">
-        <v>0</v>
-      </c>
-      <c r="G7" s="5">
+      <c r="C7" s="6"/>
+      <c r="D7" s="6">
+        <v>0</v>
+      </c>
+      <c r="E7" s="19">
+        <v>0</v>
+      </c>
+      <c r="F7" s="19">
+        <v>0</v>
+      </c>
+      <c r="G7" s="19">
         <v>0</v>
       </c>
       <c r="S7" s="3"/>
     </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B8" s="7" t="s">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="5">
-        <v>0</v>
-      </c>
-      <c r="F8" s="5">
-        <v>0</v>
-      </c>
-      <c r="G8" s="5">
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="19">
+        <v>0</v>
+      </c>
+      <c r="F8" s="19">
+        <v>0</v>
+      </c>
+      <c r="G8" s="19">
         <v>0</v>
       </c>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B9" s="12" t="s">
+    <row r="9" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B9" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5">
-        <v>0</v>
-      </c>
-      <c r="G9" s="5">
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="19">
+        <v>0</v>
+      </c>
+      <c r="F9" s="19">
+        <v>0</v>
+      </c>
+      <c r="G9" s="19">
         <v>0</v>
       </c>
       <c r="L9" s="4"/>
@@ -788,214 +793,214 @@
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
     </row>
-    <row r="10" spans="2:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="12" t="s">
+    <row r="10" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
       <c r="P10" s="3"/>
       <c r="S10" s="3"/>
     </row>
-    <row r="11" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B11" s="7" t="s">
+    <row r="11" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="7">
-        <v>0</v>
-      </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="5">
-        <v>0</v>
-      </c>
-      <c r="F11" s="5">
-        <v>0</v>
-      </c>
-      <c r="G11" s="5">
+      <c r="C11" s="6">
+        <v>0</v>
+      </c>
+      <c r="D11" s="8"/>
+      <c r="E11" s="19">
+        <v>0</v>
+      </c>
+      <c r="F11" s="19">
+        <v>0</v>
+      </c>
+      <c r="G11" s="19">
         <v>0</v>
       </c>
       <c r="P11" s="3"/>
       <c r="S11" s="3"/>
     </row>
-    <row r="12" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B12" s="7" t="s">
+    <row r="12" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B12" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7">
-        <v>0</v>
-      </c>
-      <c r="E12" s="5">
-        <v>0</v>
-      </c>
-      <c r="F12" s="5">
-        <v>0</v>
-      </c>
-      <c r="G12" s="5">
+      <c r="C12" s="6"/>
+      <c r="D12" s="6">
+        <v>0</v>
+      </c>
+      <c r="E12" s="19">
+        <v>0</v>
+      </c>
+      <c r="F12" s="19">
+        <v>0</v>
+      </c>
+      <c r="G12" s="19">
         <v>0</v>
       </c>
       <c r="P12" s="3"/>
       <c r="S12" s="3"/>
     </row>
-    <row r="13" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B13" s="7" t="s">
+    <row r="13" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B13" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="5">
-        <v>0</v>
-      </c>
-      <c r="F13" s="5">
-        <v>0</v>
-      </c>
-      <c r="G13" s="5">
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="19">
+        <v>0</v>
+      </c>
+      <c r="F13" s="19">
+        <v>0</v>
+      </c>
+      <c r="G13" s="19">
         <v>0</v>
       </c>
       <c r="P13" s="4"/>
       <c r="S13" s="3"/>
     </row>
-    <row r="14" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B14" s="12" t="s">
+    <row r="14" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B14" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="5">
-        <v>0</v>
-      </c>
-      <c r="F14" s="5">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5">
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="19">
+        <v>0</v>
+      </c>
+      <c r="F14" s="19">
+        <v>0</v>
+      </c>
+      <c r="G14" s="19">
         <v>0</v>
       </c>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" spans="2:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="12" t="s">
+    <row r="15" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
       <c r="P15" s="3"/>
       <c r="S15" s="3"/>
     </row>
-    <row r="16" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B16" s="7" t="s">
+    <row r="16" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="5">
-        <v>0</v>
-      </c>
-      <c r="F16" s="5">
-        <v>0</v>
-      </c>
-      <c r="G16" s="5">
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="19">
+        <v>0</v>
+      </c>
+      <c r="F16" s="19">
+        <v>0</v>
+      </c>
+      <c r="G16" s="19">
         <v>0</v>
       </c>
       <c r="P16" s="3"/>
       <c r="S16" s="3"/>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B17" s="7" t="s">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="5">
-        <v>0</v>
-      </c>
-      <c r="F17" s="5">
-        <v>0</v>
-      </c>
-      <c r="G17" s="5">
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="19">
+        <v>0</v>
+      </c>
+      <c r="F17" s="19">
+        <v>0</v>
+      </c>
+      <c r="G17" s="19">
         <v>0</v>
       </c>
       <c r="L17" s="4"/>
       <c r="P17" s="3"/>
       <c r="S17" s="3"/>
     </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B18" s="7" t="s">
+    <row r="18" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B18" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="5">
-        <v>0</v>
-      </c>
-      <c r="F18" s="5">
-        <v>0</v>
-      </c>
-      <c r="G18" s="5">
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="19">
+        <v>0</v>
+      </c>
+      <c r="F18" s="19">
+        <v>0</v>
+      </c>
+      <c r="G18" s="19">
         <v>0</v>
       </c>
       <c r="L18" s="4"/>
       <c r="P18" s="4"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B19" s="7" t="s">
+    <row r="19" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B19" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="5">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5">
-        <v>0</v>
-      </c>
-      <c r="G19" s="5">
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="19">
+        <v>0</v>
+      </c>
+      <c r="F19" s="19">
+        <v>0</v>
+      </c>
+      <c r="G19" s="19">
         <v>0</v>
       </c>
       <c r="L19" s="4"/>
       <c r="P19" s="3"/>
       <c r="S19" s="3"/>
     </row>
-    <row r="20" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B20" s="7" t="s">
+    <row r="20" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B20" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="5">
-        <v>0</v>
-      </c>
-      <c r="F20" s="5">
-        <v>0</v>
-      </c>
-      <c r="G20" s="5">
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="19">
+        <v>0</v>
+      </c>
+      <c r="F20" s="19">
+        <v>0</v>
+      </c>
+      <c r="G20" s="19">
         <v>0</v>
       </c>
       <c r="L20" s="4"/>
       <c r="P20" s="3"/>
       <c r="S20" s="3"/>
     </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B21" s="12" t="s">
+    <row r="21" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B21" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="5">
-        <v>0</v>
-      </c>
-      <c r="F21" s="5">
-        <v>0</v>
-      </c>
-      <c r="G21" s="5">
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="19">
+        <v>0</v>
+      </c>
+      <c r="F21" s="19">
+        <v>0</v>
+      </c>
+      <c r="G21" s="19">
         <v>0</v>
       </c>
       <c r="L21" s="4"/>
@@ -1005,56 +1010,56 @@
       <c r="P21" s="3"/>
       <c r="S21" s="3"/>
     </row>
-    <row r="22" spans="2:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="10" t="s">
+    <row r="22" spans="2:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
       <c r="P22" s="3"/>
       <c r="S22" s="3"/>
     </row>
-    <row r="23" spans="2:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="7" t="s">
+    <row r="23" spans="2:19" ht="18.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C23" s="7">
-        <v>0</v>
-      </c>
-      <c r="D23" s="7"/>
-      <c r="E23" s="5">
-        <v>0</v>
-      </c>
-      <c r="F23" s="5">
-        <v>0</v>
-      </c>
-      <c r="G23" s="5">
+      <c r="C23" s="6">
+        <v>0</v>
+      </c>
+      <c r="D23" s="6"/>
+      <c r="E23" s="19">
+        <v>0</v>
+      </c>
+      <c r="F23" s="19">
+        <v>0</v>
+      </c>
+      <c r="G23" s="19">
         <v>0</v>
       </c>
       <c r="H23" s="4"/>
       <c r="P23" s="4"/>
       <c r="S23" s="3"/>
     </row>
-    <row r="24" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B24" s="7" t="s">
+    <row r="24" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B24" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="7">
-        <v>0</v>
-      </c>
-      <c r="D24" s="7">
-        <v>0</v>
-      </c>
-      <c r="E24" s="5">
-        <v>0</v>
-      </c>
-      <c r="F24" s="5">
-        <v>0</v>
-      </c>
-      <c r="G24" s="5">
+      <c r="C24" s="6">
+        <v>0</v>
+      </c>
+      <c r="D24" s="6">
+        <v>0</v>
+      </c>
+      <c r="E24" s="19">
+        <v>0</v>
+      </c>
+      <c r="F24" s="19">
+        <v>0</v>
+      </c>
+      <c r="G24" s="19">
         <v>0</v>
       </c>
       <c r="H24" s="4"/>
@@ -1062,19 +1067,19 @@
       <c r="P24" s="3"/>
       <c r="S24" s="3"/>
     </row>
-    <row r="25" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B25" s="9" t="s">
+    <row r="25" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B25" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="8">
-        <v>0</v>
-      </c>
-      <c r="F25" s="8">
-        <v>0</v>
-      </c>
-      <c r="G25" s="8">
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="20">
+        <v>0</v>
+      </c>
+      <c r="F25" s="20">
+        <v>0</v>
+      </c>
+      <c r="G25" s="20">
         <v>0</v>
       </c>
       <c r="H25" s="4"/>
@@ -1082,19 +1087,19 @@
       <c r="P25" s="3"/>
       <c r="S25" s="3"/>
     </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B26" s="7" t="s">
+    <row r="26" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B26" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="5">
-        <v>0</v>
-      </c>
-      <c r="F26" s="5">
-        <v>0</v>
-      </c>
-      <c r="G26" s="5">
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="19">
+        <v>0</v>
+      </c>
+      <c r="F26" s="19">
+        <v>0</v>
+      </c>
+      <c r="G26" s="19">
         <v>0</v>
       </c>
       <c r="H26" s="4"/>
@@ -1104,98 +1109,98 @@
       <c r="P26" s="3"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B27" s="7" t="s">
+    <row r="27" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B27" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C27" s="7">
-        <v>0</v>
-      </c>
-      <c r="D27" s="7">
-        <v>0</v>
-      </c>
-      <c r="E27" s="5">
-        <v>0</v>
-      </c>
-      <c r="F27" s="5">
-        <v>0</v>
-      </c>
-      <c r="G27" s="5">
+      <c r="C27" s="6">
+        <v>0</v>
+      </c>
+      <c r="D27" s="6">
+        <v>0</v>
+      </c>
+      <c r="E27" s="19">
+        <v>0</v>
+      </c>
+      <c r="F27" s="19">
+        <v>0</v>
+      </c>
+      <c r="G27" s="19">
         <v>0</v>
       </c>
       <c r="H27" s="4"/>
       <c r="P27" s="3"/>
       <c r="S27" s="3"/>
     </row>
-    <row r="28" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B28" s="7" t="s">
+    <row r="28" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B28" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C28" s="7">
-        <v>0</v>
-      </c>
-      <c r="D28" s="7">
-        <v>0</v>
-      </c>
-      <c r="E28" s="5">
-        <v>0</v>
-      </c>
-      <c r="F28" s="5">
-        <v>0</v>
-      </c>
-      <c r="G28" s="5">
+      <c r="C28" s="6">
+        <v>0</v>
+      </c>
+      <c r="D28" s="6">
+        <v>0</v>
+      </c>
+      <c r="E28" s="19">
+        <v>0</v>
+      </c>
+      <c r="F28" s="19">
+        <v>0</v>
+      </c>
+      <c r="G28" s="19">
         <v>0</v>
       </c>
       <c r="H28" s="4"/>
       <c r="P28" s="3"/>
       <c r="S28" s="3"/>
     </row>
-    <row r="29" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B29" s="7" t="s">
+    <row r="29" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B29" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C29" s="7">
-        <v>0</v>
-      </c>
-      <c r="D29" s="7">
-        <v>0</v>
-      </c>
-      <c r="E29" s="5">
-        <v>0</v>
-      </c>
-      <c r="F29" s="5">
-        <v>0</v>
-      </c>
-      <c r="G29" s="5">
+      <c r="C29" s="6">
+        <v>0</v>
+      </c>
+      <c r="D29" s="6">
+        <v>0</v>
+      </c>
+      <c r="E29" s="19">
+        <v>0</v>
+      </c>
+      <c r="F29" s="19">
+        <v>0</v>
+      </c>
+      <c r="G29" s="19">
         <v>0</v>
       </c>
       <c r="H29" s="4"/>
       <c r="P29" s="3"/>
       <c r="S29" s="3"/>
     </row>
-    <row r="30" spans="2:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="C30" s="7">
-        <v>0</v>
-      </c>
-      <c r="D30" s="6">
-        <v>0</v>
-      </c>
-      <c r="E30" s="5">
-        <v>0</v>
-      </c>
-      <c r="F30" s="5">
-        <v>0</v>
-      </c>
-      <c r="G30" s="5">
+    <row r="30" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C30" s="6">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5">
+        <v>0</v>
+      </c>
+      <c r="E30" s="19">
+        <v>0</v>
+      </c>
+      <c r="F30" s="19">
+        <v>0</v>
+      </c>
+      <c r="G30" s="19">
         <v>0</v>
       </c>
       <c r="H30" s="4"/>
       <c r="P30" s="4"/>
     </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
@@ -1206,7 +1211,7 @@
       <c r="L31" s="4"/>
       <c r="P31" s="3"/>
     </row>
-    <row r="32" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
@@ -1220,18 +1225,18 @@
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
     </row>
-    <row r="33" spans="5:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E33" s="2"/>
       <c r="L33" s="4"/>
       <c r="P33" s="3"/>
     </row>
-    <row r="35" spans="5:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E35" s="2"/>
     </row>
-    <row r="37" spans="5:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="5:16" x14ac:dyDescent="0.2">
       <c r="F37" s="2"/>
     </row>
-    <row r="38" spans="5:16" x14ac:dyDescent="0.3">
+    <row r="38" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E38" s="2"/>
     </row>
   </sheetData>
@@ -1240,5 +1245,6 @@
     <mergeCell ref="B22:G22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="86" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[refs #36200] Approval Summary format enforcement.
</commit_message>
<xml_diff>
--- a/core/api/export/templates/approval_summary_template.xlsx
+++ b/core/api/export/templates/approval_summary_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Work/edw/ors-multilateralfund/core/api/export/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE109C0F-ECC6-1F41-8653-EAE05C0DB67E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED211EB-01A7-B24F-AF6F-208CC8E29650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="2800" windowWidth="28480" windowHeight="15420" xr2:uid="{EFCB9BCD-D7D4-4B7E-959C-9F2ED12FB513}"/>
+    <workbookView xWindow="760" yWindow="2800" windowWidth="28480" windowHeight="15420" xr2:uid="{EFCB9BCD-D7D4-4B7E-959C-9F2ED12FB513}"/>
   </bookViews>
   <sheets>
     <sheet name="Approval summary" sheetId="2" r:id="rId1"/>
@@ -132,7 +132,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="#,##0;[Red]\-&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,13 +166,6 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -271,18 +264,14 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -290,7 +279,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -305,6 +294,10 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -646,7 +639,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" ht="23.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="16" t="s">
         <v>26</v>
       </c>
       <c r="C1" s="4"/>
@@ -656,65 +649,65 @@
       <c r="G1" s="4"/>
     </row>
     <row r="2" spans="2:19" ht="18.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="2:19" ht="25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="15"/>
-      <c r="C3" s="14" t="s">
+      <c r="B3" s="13"/>
+      <c r="C3" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="10" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="4" spans="2:19" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
       <c r="S4" s="3"/>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="6">
-        <v>0</v>
-      </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="19">
-        <v>0</v>
-      </c>
-      <c r="F5" s="19">
-        <v>0</v>
-      </c>
-      <c r="G5" s="19">
+      <c r="C5" s="22">
+        <v>0</v>
+      </c>
+      <c r="D5" s="22"/>
+      <c r="E5" s="17">
+        <v>0</v>
+      </c>
+      <c r="F5" s="17">
+        <v>0</v>
+      </c>
+      <c r="G5" s="17">
         <v>0</v>
       </c>
       <c r="S5" s="3"/>
@@ -723,15 +716,15 @@
       <c r="B6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="19">
-        <v>0</v>
-      </c>
-      <c r="F6" s="19">
-        <v>0</v>
-      </c>
-      <c r="G6" s="19">
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="17">
+        <v>0</v>
+      </c>
+      <c r="F6" s="17">
+        <v>0</v>
+      </c>
+      <c r="G6" s="17">
         <v>0</v>
       </c>
       <c r="S6" s="3"/>
@@ -740,17 +733,17 @@
       <c r="B7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6">
-        <v>0</v>
-      </c>
-      <c r="E7" s="19">
-        <v>0</v>
-      </c>
-      <c r="F7" s="19">
-        <v>0</v>
-      </c>
-      <c r="G7" s="19">
+      <c r="C7" s="22"/>
+      <c r="D7" s="22">
+        <v>0</v>
+      </c>
+      <c r="E7" s="17">
+        <v>0</v>
+      </c>
+      <c r="F7" s="17">
+        <v>0</v>
+      </c>
+      <c r="G7" s="17">
         <v>0</v>
       </c>
       <c r="S7" s="3"/>
@@ -759,32 +752,32 @@
       <c r="B8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="19">
-        <v>0</v>
-      </c>
-      <c r="F8" s="19">
-        <v>0</v>
-      </c>
-      <c r="G8" s="19">
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="17">
+        <v>0</v>
+      </c>
+      <c r="F8" s="17">
+        <v>0</v>
+      </c>
+      <c r="G8" s="17">
         <v>0</v>
       </c>
       <c r="S8" s="4"/>
     </row>
     <row r="9" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="19">
-        <v>0</v>
-      </c>
-      <c r="F9" s="19">
-        <v>0</v>
-      </c>
-      <c r="G9" s="19">
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="17">
+        <v>0</v>
+      </c>
+      <c r="F9" s="17">
+        <v>0</v>
+      </c>
+      <c r="G9" s="17">
         <v>0</v>
       </c>
       <c r="L9" s="4"/>
@@ -794,14 +787,14 @@
       <c r="P9" s="3"/>
     </row>
     <row r="10" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
       <c r="P10" s="3"/>
       <c r="S10" s="3"/>
     </row>
@@ -809,17 +802,17 @@
       <c r="B11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="6">
-        <v>0</v>
-      </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="19">
-        <v>0</v>
-      </c>
-      <c r="F11" s="19">
-        <v>0</v>
-      </c>
-      <c r="G11" s="19">
+      <c r="C11" s="22">
+        <v>0</v>
+      </c>
+      <c r="D11" s="22"/>
+      <c r="E11" s="17">
+        <v>0</v>
+      </c>
+      <c r="F11" s="17">
+        <v>0</v>
+      </c>
+      <c r="G11" s="17">
         <v>0</v>
       </c>
       <c r="P11" s="3"/>
@@ -829,17 +822,17 @@
       <c r="B12" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6">
-        <v>0</v>
-      </c>
-      <c r="E12" s="19">
-        <v>0</v>
-      </c>
-      <c r="F12" s="19">
-        <v>0</v>
-      </c>
-      <c r="G12" s="19">
+      <c r="C12" s="22"/>
+      <c r="D12" s="22">
+        <v>0</v>
+      </c>
+      <c r="E12" s="17">
+        <v>0</v>
+      </c>
+      <c r="F12" s="17">
+        <v>0</v>
+      </c>
+      <c r="G12" s="17">
         <v>0</v>
       </c>
       <c r="P12" s="3"/>
@@ -849,46 +842,46 @@
       <c r="B13" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="19">
-        <v>0</v>
-      </c>
-      <c r="F13" s="19">
-        <v>0</v>
-      </c>
-      <c r="G13" s="19">
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="17">
+        <v>0</v>
+      </c>
+      <c r="F13" s="17">
+        <v>0</v>
+      </c>
+      <c r="G13" s="17">
         <v>0</v>
       </c>
       <c r="P13" s="4"/>
       <c r="S13" s="3"/>
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="19">
-        <v>0</v>
-      </c>
-      <c r="F14" s="19">
-        <v>0</v>
-      </c>
-      <c r="G14" s="19">
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="17">
+        <v>0</v>
+      </c>
+      <c r="F14" s="17">
+        <v>0</v>
+      </c>
+      <c r="G14" s="17">
         <v>0</v>
       </c>
       <c r="S14" s="4"/>
     </row>
     <row r="15" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
       <c r="P15" s="3"/>
@@ -898,15 +891,15 @@
       <c r="B16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="19">
-        <v>0</v>
-      </c>
-      <c r="F16" s="19">
-        <v>0</v>
-      </c>
-      <c r="G16" s="19">
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="17">
+        <v>0</v>
+      </c>
+      <c r="F16" s="17">
+        <v>0</v>
+      </c>
+      <c r="G16" s="17">
         <v>0</v>
       </c>
       <c r="P16" s="3"/>
@@ -916,15 +909,15 @@
       <c r="B17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="19">
-        <v>0</v>
-      </c>
-      <c r="F17" s="19">
-        <v>0</v>
-      </c>
-      <c r="G17" s="19">
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="17">
+        <v>0</v>
+      </c>
+      <c r="F17" s="17">
+        <v>0</v>
+      </c>
+      <c r="G17" s="17">
         <v>0</v>
       </c>
       <c r="L17" s="4"/>
@@ -935,15 +928,15 @@
       <c r="B18" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="19">
-        <v>0</v>
-      </c>
-      <c r="F18" s="19">
-        <v>0</v>
-      </c>
-      <c r="G18" s="19">
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="17">
+        <v>0</v>
+      </c>
+      <c r="F18" s="17">
+        <v>0</v>
+      </c>
+      <c r="G18" s="17">
         <v>0</v>
       </c>
       <c r="L18" s="4"/>
@@ -954,15 +947,15 @@
       <c r="B19" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="19">
-        <v>0</v>
-      </c>
-      <c r="F19" s="19">
-        <v>0</v>
-      </c>
-      <c r="G19" s="19">
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="17">
+        <v>0</v>
+      </c>
+      <c r="F19" s="17">
+        <v>0</v>
+      </c>
+      <c r="G19" s="17">
         <v>0</v>
       </c>
       <c r="L19" s="4"/>
@@ -973,15 +966,15 @@
       <c r="B20" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="19">
-        <v>0</v>
-      </c>
-      <c r="F20" s="19">
-        <v>0</v>
-      </c>
-      <c r="G20" s="19">
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="17">
+        <v>0</v>
+      </c>
+      <c r="F20" s="17">
+        <v>0</v>
+      </c>
+      <c r="G20" s="17">
         <v>0</v>
       </c>
       <c r="L20" s="4"/>
@@ -989,18 +982,18 @@
       <c r="S20" s="3"/>
     </row>
     <row r="21" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="19">
-        <v>0</v>
-      </c>
-      <c r="F21" s="19">
-        <v>0</v>
-      </c>
-      <c r="G21" s="19">
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="17">
+        <v>0</v>
+      </c>
+      <c r="F21" s="17">
+        <v>0</v>
+      </c>
+      <c r="G21" s="17">
         <v>0</v>
       </c>
       <c r="L21" s="4"/>
@@ -1011,14 +1004,14 @@
       <c r="S21" s="3"/>
     </row>
     <row r="22" spans="2:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
       <c r="P22" s="3"/>
       <c r="S22" s="3"/>
     </row>
@@ -1030,13 +1023,13 @@
         <v>0</v>
       </c>
       <c r="D23" s="6"/>
-      <c r="E23" s="19">
-        <v>0</v>
-      </c>
-      <c r="F23" s="19">
-        <v>0</v>
-      </c>
-      <c r="G23" s="19">
+      <c r="E23" s="17">
+        <v>0</v>
+      </c>
+      <c r="F23" s="17">
+        <v>0</v>
+      </c>
+      <c r="G23" s="17">
         <v>0</v>
       </c>
       <c r="H23" s="4"/>
@@ -1053,13 +1046,13 @@
       <c r="D24" s="6">
         <v>0</v>
       </c>
-      <c r="E24" s="19">
-        <v>0</v>
-      </c>
-      <c r="F24" s="19">
-        <v>0</v>
-      </c>
-      <c r="G24" s="19">
+      <c r="E24" s="17">
+        <v>0</v>
+      </c>
+      <c r="F24" s="17">
+        <v>0</v>
+      </c>
+      <c r="G24" s="17">
         <v>0</v>
       </c>
       <c r="H24" s="4"/>
@@ -1073,13 +1066,13 @@
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
-      <c r="E25" s="20">
-        <v>0</v>
-      </c>
-      <c r="F25" s="20">
-        <v>0</v>
-      </c>
-      <c r="G25" s="20">
+      <c r="E25" s="18">
+        <v>0</v>
+      </c>
+      <c r="F25" s="18">
+        <v>0</v>
+      </c>
+      <c r="G25" s="18">
         <v>0</v>
       </c>
       <c r="H25" s="4"/>
@@ -1093,13 +1086,13 @@
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
-      <c r="E26" s="19">
-        <v>0</v>
-      </c>
-      <c r="F26" s="19">
-        <v>0</v>
-      </c>
-      <c r="G26" s="19">
+      <c r="E26" s="17">
+        <v>0</v>
+      </c>
+      <c r="F26" s="17">
+        <v>0</v>
+      </c>
+      <c r="G26" s="17">
         <v>0</v>
       </c>
       <c r="H26" s="4"/>
@@ -1119,13 +1112,13 @@
       <c r="D27" s="6">
         <v>0</v>
       </c>
-      <c r="E27" s="19">
-        <v>0</v>
-      </c>
-      <c r="F27" s="19">
-        <v>0</v>
-      </c>
-      <c r="G27" s="19">
+      <c r="E27" s="17">
+        <v>0</v>
+      </c>
+      <c r="F27" s="17">
+        <v>0</v>
+      </c>
+      <c r="G27" s="17">
         <v>0</v>
       </c>
       <c r="H27" s="4"/>
@@ -1142,13 +1135,13 @@
       <c r="D28" s="6">
         <v>0</v>
       </c>
-      <c r="E28" s="19">
-        <v>0</v>
-      </c>
-      <c r="F28" s="19">
-        <v>0</v>
-      </c>
-      <c r="G28" s="19">
+      <c r="E28" s="17">
+        <v>0</v>
+      </c>
+      <c r="F28" s="17">
+        <v>0</v>
+      </c>
+      <c r="G28" s="17">
         <v>0</v>
       </c>
       <c r="H28" s="4"/>
@@ -1165,13 +1158,13 @@
       <c r="D29" s="6">
         <v>0</v>
       </c>
-      <c r="E29" s="19">
-        <v>0</v>
-      </c>
-      <c r="F29" s="19">
-        <v>0</v>
-      </c>
-      <c r="G29" s="19">
+      <c r="E29" s="17">
+        <v>0</v>
+      </c>
+      <c r="F29" s="17">
+        <v>0</v>
+      </c>
+      <c r="G29" s="17">
         <v>0</v>
       </c>
       <c r="H29" s="4"/>
@@ -1188,13 +1181,13 @@
       <c r="D30" s="5">
         <v>0</v>
       </c>
-      <c r="E30" s="19">
-        <v>0</v>
-      </c>
-      <c r="F30" s="19">
-        <v>0</v>
-      </c>
-      <c r="G30" s="19">
+      <c r="E30" s="17">
+        <v>0</v>
+      </c>
+      <c r="F30" s="17">
+        <v>0</v>
+      </c>
+      <c r="G30" s="17">
         <v>0</v>
       </c>
       <c r="H30" s="4"/>

</xml_diff>

<commit_message>
[refs #36200] Approval summary: insert row in template.
</commit_message>
<xml_diff>
--- a/core/api/export/templates/approval_summary_template.xlsx
+++ b/core/api/export/templates/approval_summary_template.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Work/edw/ors-multilateralfund/core/api/export/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED211EB-01A7-B24F-AF6F-208CC8E29650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6634EA7C-EA26-A24D-A321-9F57DC8577A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="2800" windowWidth="28480" windowHeight="15420" xr2:uid="{EFCB9BCD-D7D4-4B7E-959C-9F2ED12FB513}"/>
+    <workbookView xWindow="740" yWindow="2800" windowWidth="28480" windowHeight="15420" xr2:uid="{EFCB9BCD-D7D4-4B7E-959C-9F2ED12FB513}"/>
   </bookViews>
   <sheets>
     <sheet name="Approval summary" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Approval summary'!$B$1:$G$53</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Approval summary'!$B$2:$G$54</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -288,16 +288,16 @@
     <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -617,7 +617,7 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:S38"/>
+  <dimension ref="B2:S39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="1"/>
@@ -638,86 +638,69 @@
     <col min="20" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:19" ht="23.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="16" t="s">
+    <row r="2" spans="2:19" ht="23.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="2:19" ht="18.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="15" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="2:19" ht="18.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C3" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D3" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E3" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-    </row>
-    <row r="3" spans="2:19" ht="25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="13"/>
-      <c r="C3" s="12" t="s">
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+    </row>
+    <row r="4" spans="2:19" ht="25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="13"/>
+      <c r="C4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E4" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="2:19" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="8" t="s">
+    <row r="5" spans="2:19" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="S4" s="3"/>
-    </row>
-    <row r="5" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="22">
-        <v>0</v>
-      </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="17">
-        <v>0</v>
-      </c>
-      <c r="F5" s="17">
-        <v>0</v>
-      </c>
-      <c r="G5" s="17">
-        <v>0</v>
-      </c>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
       <c r="S5" s="3"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
+        <v>14</v>
+      </c>
+      <c r="C6" s="20">
+        <v>0</v>
+      </c>
+      <c r="D6" s="20"/>
       <c r="E6" s="17">
         <v>0</v>
       </c>
@@ -731,12 +714,10 @@
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B7" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22">
-        <v>0</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
       <c r="E7" s="17">
         <v>0</v>
       </c>
@@ -750,82 +731,81 @@
     </row>
     <row r="8" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20">
+        <v>0</v>
+      </c>
+      <c r="E8" s="17">
+        <v>0</v>
+      </c>
+      <c r="F8" s="17">
+        <v>0</v>
+      </c>
+      <c r="G8" s="17">
+        <v>0</v>
+      </c>
+      <c r="S8" s="3"/>
+    </row>
+    <row r="9" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="17">
-        <v>0</v>
-      </c>
-      <c r="F8" s="17">
-        <v>0</v>
-      </c>
-      <c r="G8" s="17">
-        <v>0</v>
-      </c>
-      <c r="S8" s="4"/>
-    </row>
-    <row r="9" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="17">
+        <v>0</v>
+      </c>
+      <c r="F9" s="17">
+        <v>0</v>
+      </c>
+      <c r="G9" s="17">
+        <v>0</v>
+      </c>
+      <c r="S9" s="4"/>
+    </row>
+    <row r="10" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B10" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="17">
-        <v>0</v>
-      </c>
-      <c r="F9" s="17">
-        <v>0</v>
-      </c>
-      <c r="G9" s="17">
-        <v>0</v>
-      </c>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-    </row>
-    <row r="10" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="17">
+        <v>0</v>
+      </c>
+      <c r="F10" s="17">
+        <v>0</v>
+      </c>
+      <c r="G10" s="17">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+    </row>
+    <row r="11" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="P10" s="3"/>
-      <c r="S10" s="3"/>
-    </row>
-    <row r="11" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B11" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="22">
-        <v>0</v>
-      </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="17">
-        <v>0</v>
-      </c>
-      <c r="F11" s="17">
-        <v>0</v>
-      </c>
-      <c r="G11" s="17">
-        <v>0</v>
-      </c>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
       <c r="P11" s="3"/>
       <c r="S11" s="3"/>
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B12" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22">
-        <v>0</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C12" s="20">
+        <v>0</v>
+      </c>
+      <c r="D12" s="20"/>
       <c r="E12" s="17">
         <v>0</v>
       </c>
@@ -840,77 +820,79 @@
     </row>
     <row r="13" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20">
+        <v>0</v>
+      </c>
+      <c r="E13" s="17">
+        <v>0</v>
+      </c>
+      <c r="F13" s="17">
+        <v>0</v>
+      </c>
+      <c r="G13" s="17">
+        <v>0</v>
+      </c>
+      <c r="P13" s="3"/>
+      <c r="S13" s="3"/>
+    </row>
+    <row r="14" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B14" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="17">
-        <v>0</v>
-      </c>
-      <c r="F13" s="17">
-        <v>0</v>
-      </c>
-      <c r="G13" s="17">
-        <v>0</v>
-      </c>
-      <c r="P13" s="4"/>
-      <c r="S13" s="3"/>
-    </row>
-    <row r="14" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="17">
+        <v>0</v>
+      </c>
+      <c r="F14" s="17">
+        <v>0</v>
+      </c>
+      <c r="G14" s="17">
+        <v>0</v>
+      </c>
+      <c r="P14" s="4"/>
+      <c r="S14" s="3"/>
+    </row>
+    <row r="15" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B15" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="17">
-        <v>0</v>
-      </c>
-      <c r="F14" s="17">
-        <v>0</v>
-      </c>
-      <c r="G14" s="17">
-        <v>0</v>
-      </c>
-      <c r="S14" s="4"/>
-    </row>
-    <row r="15" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="8" t="s">
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="17">
+        <v>0</v>
+      </c>
+      <c r="F15" s="17">
+        <v>0</v>
+      </c>
+      <c r="G15" s="17">
+        <v>0</v>
+      </c>
+      <c r="S15" s="4"/>
+    </row>
+    <row r="16" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="P15" s="3"/>
-      <c r="S15" s="3"/>
-    </row>
-    <row r="16" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B16" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="17">
-        <v>0</v>
-      </c>
-      <c r="F16" s="17">
-        <v>0</v>
-      </c>
-      <c r="G16" s="17">
-        <v>0</v>
-      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
       <c r="P16" s="3"/>
       <c r="S16" s="3"/>
     </row>
     <row r="17" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B17" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
+        <v>14</v>
+      </c>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
       <c r="E17" s="17">
         <v>0</v>
       </c>
@@ -920,16 +902,15 @@
       <c r="G17" s="17">
         <v>0</v>
       </c>
-      <c r="L17" s="4"/>
       <c r="P17" s="3"/>
       <c r="S17" s="3"/>
     </row>
     <row r="18" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B18" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
+        <v>13</v>
+      </c>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
       <c r="E18" s="17">
         <v>0</v>
       </c>
@@ -940,15 +921,15 @@
         <v>0</v>
       </c>
       <c r="L18" s="4"/>
-      <c r="P18" s="4"/>
-      <c r="S18" s="4"/>
+      <c r="P18" s="3"/>
+      <c r="S18" s="3"/>
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B19" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
+        <v>12</v>
+      </c>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
       <c r="E19" s="17">
         <v>0</v>
       </c>
@@ -959,15 +940,15 @@
         <v>0</v>
       </c>
       <c r="L19" s="4"/>
-      <c r="P19" s="3"/>
-      <c r="S19" s="3"/>
+      <c r="P19" s="4"/>
+      <c r="S19" s="4"/>
     </row>
     <row r="20" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B20" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
+        <v>11</v>
+      </c>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
       <c r="E20" s="17">
         <v>0</v>
       </c>
@@ -982,11 +963,11 @@
       <c r="S20" s="3"/>
     </row>
     <row r="21" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B21" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
+      <c r="B21" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
       <c r="E21" s="17">
         <v>0</v>
       </c>
@@ -997,82 +978,81 @@
         <v>0</v>
       </c>
       <c r="L21" s="4"/>
-      <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="3"/>
       <c r="P21" s="3"/>
       <c r="S21" s="3"/>
     </row>
-    <row r="22" spans="2:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="20" t="s">
-        <v>8</v>
+    <row r="22" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B22" s="8" t="s">
+        <v>9</v>
       </c>
       <c r="C22" s="20"/>
       <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
+      <c r="E22" s="17">
+        <v>0</v>
+      </c>
+      <c r="F22" s="17">
+        <v>0</v>
+      </c>
+      <c r="G22" s="17">
+        <v>0</v>
+      </c>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="3"/>
       <c r="P22" s="3"/>
       <c r="S22" s="3"/>
     </row>
-    <row r="23" spans="2:19" ht="18.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="6" t="s">
+    <row r="23" spans="2:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
+      <c r="P23" s="3"/>
+      <c r="S23" s="3"/>
+    </row>
+    <row r="24" spans="2:19" ht="18.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C23" s="6">
-        <v>0</v>
-      </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="17">
-        <v>0</v>
-      </c>
-      <c r="F23" s="17">
-        <v>0</v>
-      </c>
-      <c r="G23" s="17">
-        <v>0</v>
-      </c>
-      <c r="H23" s="4"/>
-      <c r="P23" s="4"/>
-      <c r="S23" s="3"/>
-    </row>
-    <row r="24" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="6">
+        <v>0</v>
+      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" s="17">
+        <v>0</v>
+      </c>
+      <c r="F24" s="17">
+        <v>0</v>
+      </c>
+      <c r="G24" s="17">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="S24" s="3"/>
+    </row>
+    <row r="25" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="6">
-        <v>0</v>
-      </c>
-      <c r="D24" s="6">
-        <v>0</v>
-      </c>
-      <c r="E24" s="17">
-        <v>0</v>
-      </c>
-      <c r="F24" s="17">
-        <v>0</v>
-      </c>
-      <c r="G24" s="17">
-        <v>0</v>
-      </c>
-      <c r="H24" s="4"/>
-      <c r="L24" s="4"/>
-      <c r="P24" s="3"/>
-      <c r="S24" s="3"/>
-    </row>
-    <row r="25" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B25" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="18">
-        <v>0</v>
-      </c>
-      <c r="F25" s="18">
-        <v>0</v>
-      </c>
-      <c r="G25" s="18">
+      <c r="C25" s="6">
+        <v>0</v>
+      </c>
+      <c r="D25" s="6">
+        <v>0</v>
+      </c>
+      <c r="E25" s="17">
+        <v>0</v>
+      </c>
+      <c r="F25" s="17">
+        <v>0</v>
+      </c>
+      <c r="G25" s="17">
         <v>0</v>
       </c>
       <c r="H25" s="4"/>
@@ -1081,37 +1061,31 @@
       <c r="S25" s="3"/>
     </row>
     <row r="26" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B26" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="17">
-        <v>0</v>
-      </c>
-      <c r="F26" s="17">
-        <v>0</v>
-      </c>
-      <c r="G26" s="17">
+      <c r="B26" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="18">
+        <v>0</v>
+      </c>
+      <c r="F26" s="18">
+        <v>0</v>
+      </c>
+      <c r="G26" s="18">
         <v>0</v>
       </c>
       <c r="H26" s="4"/>
-      <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
-      <c r="O26" s="3"/>
+      <c r="L26" s="4"/>
       <c r="P26" s="3"/>
-      <c r="S26" s="4"/>
+      <c r="S26" s="3"/>
     </row>
     <row r="27" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B27" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C27" s="6">
-        <v>0</v>
-      </c>
-      <c r="D27" s="6">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
       <c r="E27" s="17">
         <v>0</v>
       </c>
@@ -1122,12 +1096,15 @@
         <v>0</v>
       </c>
       <c r="H27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="3"/>
       <c r="P27" s="3"/>
-      <c r="S27" s="3"/>
+      <c r="S27" s="4"/>
     </row>
     <row r="28" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B28" s="6" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C28" s="6">
         <v>0</v>
@@ -1150,7 +1127,7 @@
     </row>
     <row r="29" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B29" s="6" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" s="6">
         <v>0</v>
@@ -1171,14 +1148,14 @@
       <c r="P29" s="3"/>
       <c r="S29" s="3"/>
     </row>
-    <row r="30" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B30" s="6" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C30" s="6">
         <v>0</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="6">
         <v>0</v>
       </c>
       <c r="E30" s="17">
@@ -1191,18 +1168,30 @@
         <v>0</v>
       </c>
       <c r="H30" s="4"/>
-      <c r="P30" s="4"/>
-    </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
+      <c r="P30" s="3"/>
+      <c r="S30" s="3"/>
+    </row>
+    <row r="31" spans="2:19" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="6">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5">
+        <v>0</v>
+      </c>
+      <c r="E31" s="17">
+        <v>0</v>
+      </c>
+      <c r="F31" s="17">
+        <v>0</v>
+      </c>
+      <c r="G31" s="17">
+        <v>0</v>
+      </c>
       <c r="H31" s="4"/>
-      <c r="L31" s="4"/>
-      <c r="P31" s="3"/>
+      <c r="P31" s="4"/>
     </row>
     <row r="32" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B32" s="4"/>
@@ -1213,29 +1202,40 @@
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
       <c r="L32" s="4"/>
-      <c r="M32" s="4"/>
-      <c r="N32" s="4"/>
-      <c r="O32" s="3"/>
       <c r="P32" s="3"/>
     </row>
-    <row r="33" spans="5:16" x14ac:dyDescent="0.2">
-      <c r="E33" s="2"/>
+    <row r="33" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
       <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="3"/>
       <c r="P33" s="3"/>
     </row>
-    <row r="35" spans="5:16" x14ac:dyDescent="0.2">
-      <c r="E35" s="2"/>
-    </row>
-    <row r="37" spans="5:16" x14ac:dyDescent="0.2">
-      <c r="F37" s="2"/>
-    </row>
-    <row r="38" spans="5:16" x14ac:dyDescent="0.2">
-      <c r="E38" s="2"/>
+    <row r="34" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="E34" s="2"/>
+      <c r="L34" s="4"/>
+      <c r="P34" s="3"/>
+    </row>
+    <row r="36" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="E36" s="2"/>
+    </row>
+    <row r="38" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="F38" s="2"/>
+    </row>
+    <row r="39" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="E39" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="B23:G23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="86" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>